<commit_message>
LiveOps page: real pricing, battle pass progression, updated art rates and crafting
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDtWPhrTtCTobbmqQj54pj
</commit_message>
<xml_diff>
--- a/games/Rogue_Deck_LiveOps_Economy.xlsx
+++ b/games/Rogue_Deck_LiveOps_Economy.xlsx
@@ -12,9 +12,10 @@
     <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Profiles" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Monetization" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Pack Odds" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Crafting" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Collection Sim" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Battle Pass" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Pack Odds" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Crafting" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Collection Sim" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="188">
   <si>
     <t xml:space="preserve">Rogue Deck – LiveOps Economy Model</t>
   </si>
@@ -61,7 +62,13 @@
     <t xml:space="preserve">Monetization</t>
   </si>
   <si>
-    <t xml:space="preserve">Gem bundles, price per pack, and offer value.</t>
+    <t xml:space="preserve">Gem tiers, first-purchase double, Daily Packs deals, battle pass tiers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XP per match and the level each profile reaches in a season.</t>
   </si>
   <si>
     <t xml:space="preserve">Pack Odds</t>
@@ -73,7 +80,7 @@
     <t xml:space="preserve">Crafting</t>
   </si>
   <si>
-    <t xml:space="preserve">Dismantle and craft values per rarity.</t>
+    <t xml:space="preserve">Dismantle and craft values per rarity, nerf refunds.</t>
   </si>
   <si>
     <t xml:space="preserve">Collection Sim</t>
@@ -217,16 +224,16 @@
     <t xml:space="preserve">"Play 1 match"</t>
   </si>
   <si>
-    <t xml:space="preserve">Daily Pack Pass: packs per day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deferred: 1 pack per day for 30 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daily Pack Pass: length</t>
-  </si>
-  <si>
-    <t xml:space="preserve">days</t>
+    <t xml:space="preserve">Daily Packs deal: packs per day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deferred: max 1 pack claimed per day, unclaimed days never expire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily Packs deal: packs (Tier 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$19.99 tier</t>
   </si>
   <si>
     <t xml:space="preserve">Weeks per month</t>
@@ -316,79 +323,148 @@
     <t xml:space="preserve">Paying player: + premium pass packs</t>
   </si>
   <si>
-    <t xml:space="preserve">Paying player: + Daily Pack Pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gem bundle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price (€)</t>
+    <t xml:space="preserve">Paying player: + Daily Packs (30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base rate ($ per 100 gems)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pack price (gems)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gem tier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price ($)</t>
   </si>
   <si>
     <t xml:space="preserve">Gems</t>
   </si>
   <si>
-    <t xml:space="preserve">Bonus vs. base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Packs (at 100 gems)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">€ per pack</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pack price in gems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Large</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Huge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offer</t>
+    <t xml:space="preserve">Free gems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ per 100 gems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$ per pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First purchase: gems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First purchase: $ per 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tier 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First purchase = "First-Time Double": double gems on a player's first purchase of each tier.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daily Packs deal</t>
   </si>
   <si>
     <t xml:space="preserve">Packs</t>
   </si>
   <si>
-    <t xml:space="preserve">Other contents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discount vs. Small bundle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daily Pack Pass (1 pack/day, 30 days)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deferred: must log in on 30 days</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Season pass – premium track</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 art-upgrade tokens, cosmetics</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Starter deck (fixed cards, default art)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">52 fixed cards ≈ 10 packs worth, no randomness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Launch bundle (limited)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Card back, 500 crafting materials</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Starter deck "packs" = 52 cards / 5 cards per pack, rounded. Prices are assumptions for a mid-range F2P card game.</t>
+    <t xml:space="preserve">Discount vs. Tier 1 pack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 pack can be claimed per day; unclaimed days do not expire. A player can own at most 2 deals; the second starts automatically when the first runs out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level jump</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contents</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gems, packs, crafting mats, cosmetic vouchers, season cosmetics (~$30 value)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Epic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium + 15 levels + exclusive cosmetic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legendary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Premium + 30 levels + exclusive cosmetic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battle passes can only be bought with money, not earned gems. Upgrades between tiers cost only the difference.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XP per level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PvP win XP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surrender earns no loss XP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PvP loss XP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XP per active minute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Match length (min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From Assumptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avg XP per match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XP to finish the pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches / season</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XP / season</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level reached</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level with Epic (+15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level with Legendary (+30)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Levels above 50 repeat rewards. PvE matches earn reduced XP depending on difficulty (not modelled).</t>
   </si>
   <si>
     <t xml:space="preserve">Rarity</t>
@@ -412,12 +488,6 @@
     <t xml:space="preserve">Rare</t>
   </si>
   <si>
-    <t xml:space="preserve">Epic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legendary</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total</t>
   </si>
   <si>
@@ -454,10 +524,10 @@
     <t xml:space="preserve">Legendary cards per pack</t>
   </si>
   <si>
-    <t xml:space="preserve">Dismantle (materials)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Craft cost (materials)</t>
+    <t xml:space="preserve">Dismantle (fragments)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Craft cost (fragments)</t>
   </si>
   <si>
     <t xml:space="preserve">Dismantles per craft</t>
@@ -472,15 +542,15 @@
     <t xml:space="preserve">Crafted cards always get the Default art. Higher art tiers only come from packs, events and art-upgrade tokens, which keeps packs relevant.</t>
   </si>
   <si>
+    <t xml:space="preserve">Nerf refund: dismantling a nerfed card returns its full craft cost.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Monte Carlo simulation (Python, 300 runs per profile). Static output – does not recalculate.</t>
   </si>
   <si>
     <t xml:space="preserve">Effects = all 61 effect variants owned (35 card + 26 Rogue). Artworks = all 312 artworks owned (52 playing cards x 4 + 26 Rogue x 4).</t>
   </si>
   <si>
-    <t xml:space="preserve">Profile</t>
-  </si>
-  <si>
     <t xml:space="preserve">Packs/month</t>
   </si>
   <si>
@@ -520,7 +590,7 @@
     <t xml:space="preserve">Month 6 artworks</t>
   </si>
   <si>
-    <t xml:space="preserve">Engaged + premium pass + Daily Pack Pass</t>
+    <t xml:space="preserve">Engaged + premium pass + Daily Packs</t>
   </si>
 </sst>
 </file>
@@ -534,7 +604,7 @@
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="#,##0"/>
     <numFmt numFmtId="169" formatCode="0.00"/>
-    <numFmt numFmtId="170" formatCode="\€0.00"/>
+    <numFmt numFmtId="170" formatCode="\$0.00"/>
     <numFmt numFmtId="171" formatCode="General"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
     <numFmt numFmtId="173" formatCode="0\x"/>
@@ -666,7 +736,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -719,11 +789,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -735,11 +805,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="172" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -999,7 +1077,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1099,26 +1177,34 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="A16" s="3"/>
       <c r="B16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1147,296 +1233,298 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>15</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B3" s="6" t="n">
         <v>0.5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>10</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>10</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>10</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>15</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>25</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B16" s="5" t="n">
         <v>3</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B17" s="5" t="n">
         <v>12</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>150</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B20" s="5" t="n">
         <v>1</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B21" s="5" t="n">
         <v>30</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D21" s="2"/>
+        <v>50</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1464,24 +1552,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>10</v>
@@ -1498,7 +1586,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>2</v>
@@ -1515,7 +1603,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>2</v>
@@ -1532,7 +1620,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B5" s="6" t="n">
         <v>0</v>
@@ -1549,7 +1637,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="6" t="n">
         <v>0.25</v>
@@ -1566,7 +1654,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>0</v>
@@ -1583,7 +1671,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B8" s="6" t="n">
         <v>0.4</v>
@@ -1607,24 +1695,24 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B11" s="7" t="n">
         <f aca="false">B2*B3*Assumptions!$B$2/60</f>
@@ -1645,7 +1733,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">Assumptions!$B$3*Assumptions!$B$4+(1-Assumptions!$B$3)*Assumptions!$B$5</f>
@@ -1666,7 +1754,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">MIN(B3*B12,Assumptions!$B$6)</f>
@@ -1687,7 +1775,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B14" s="10" t="n">
         <f aca="false">B2*B13</f>
@@ -1708,7 +1796,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B15" s="10" t="n">
         <f aca="false">B2*(MIN(B4,Assumptions!$B$7)*Assumptions!$B$8+B5*Assumptions!$B$9)</f>
@@ -1729,7 +1817,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">Assumptions!$B$22*B6*Assumptions!$B$10*Assumptions!$B$11+B7*Assumptions!$B$13*Assumptions!$B$14</f>
@@ -1750,7 +1838,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B17" s="10" t="n">
         <f aca="false">B14+B15+B16</f>
@@ -1771,7 +1859,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">B17/Assumptions!$B$18</f>
@@ -1792,7 +1880,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B19" s="7" t="n">
         <f aca="false">B2*Assumptions!$B$19</f>
@@ -1813,7 +1901,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">Assumptions!$B$22*B6*Assumptions!$B$12+B7*Assumptions!$B$15+B8*Assumptions!$B$16</f>
@@ -1834,7 +1922,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B21" s="7" t="n">
         <f aca="false">B18+B19+B20</f>
@@ -1855,7 +1943,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">IF(B2&gt;0,B21/B2,0)</f>
@@ -1876,7 +1964,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">B21+Assumptions!$B$17</f>
@@ -1897,7 +1985,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B24" s="7" t="n">
         <f aca="false">B23+Assumptions!$B$20*Assumptions!$B$21</f>
@@ -1932,291 +2020,300 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="B1" s="12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>102</v>
-      </c>
+      <c r="E1" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1" s="2"/>
       <c r="G1" s="2"/>
-      <c r="H1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="I1" s="5" t="n">
-        <v>100</v>
-      </c>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" s="12" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>500</v>
-      </c>
-      <c r="D2" s="13" t="n">
-        <f aca="false">C2/(B2/$B$2*$C$2)-1</f>
-        <v>0</v>
-      </c>
-      <c r="E2" s="14" t="n">
-        <f aca="false">C2/$I$1</f>
-        <v>5</v>
-      </c>
-      <c r="F2" s="15" t="n">
-        <f aca="false">B2/E2</f>
-        <v>0.998</v>
-      </c>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B3" s="12" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>1100</v>
-      </c>
-      <c r="D3" s="13" t="n">
-        <f aca="false">C3/(B3/$B$2*$C$2)-1</f>
-        <v>0.0988988988988988</v>
-      </c>
-      <c r="E3" s="14" t="n">
-        <f aca="false">C3/$I$1</f>
-        <v>11</v>
-      </c>
-      <c r="F3" s="15" t="n">
-        <f aca="false">B3/E3</f>
-        <v>0.908181818181818</v>
-      </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="F3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B4" s="12" t="n">
-        <v>19.99</v>
+        <v>1.5</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>2400</v>
+        <v>100</v>
       </c>
       <c r="D4" s="13" t="n">
-        <f aca="false">C4/(B4/$B$2*$C$2)-1</f>
-        <v>0.198199099549775</v>
+        <f aca="false">C4-ROUND(B4/$B$1*100,0)</f>
+        <v>0</v>
       </c>
       <c r="E4" s="14" t="n">
-        <f aca="false">C4/$I$1</f>
-        <v>24</v>
+        <f aca="false">1-F4/$B$1</f>
+        <v>0</v>
       </c>
       <c r="F4" s="15" t="n">
-        <f aca="false">B4/E4</f>
-        <v>0.832916666666667</v>
-      </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+        <f aca="false">B4/C4*100</f>
+        <v>1.5</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <f aca="false">F4*$E$1/100</f>
+        <v>1.5</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="I4" s="15" t="n">
+        <f aca="false">B4/H4*100</f>
+        <v>0.75</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B5" s="12" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>385</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <f aca="false">C5-ROUND(B5/$B$1*100,0)</f>
+        <v>52</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <f aca="false">1-F5/$B$1</f>
+        <v>0.135930735930736</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <f aca="false">B5/C5*100</f>
+        <v>1.2961038961039</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <f aca="false">F5*$E$1/100</f>
+        <v>1.2961038961039</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>770</v>
+      </c>
+      <c r="I5" s="15" t="n">
+        <f aca="false">B5/H5*100</f>
+        <v>0.648051948051948</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>835</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <f aca="false">C6-ROUND(B6/$B$1*100,0)</f>
+        <v>169</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <f aca="false">1-F6/$B$1</f>
+        <v>0.202395209580838</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <f aca="false">B6/C6*100</f>
+        <v>1.19640718562874</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <f aca="false">F6*$E$1/100</f>
+        <v>1.19640718562874</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1670</v>
+      </c>
+      <c r="I6" s="15" t="n">
+        <f aca="false">B6/H6*100</f>
+        <v>0.598203592814371</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="12" t="n">
         <v>49.99</v>
       </c>
-      <c r="C5" s="5" t="n">
-        <v>6500</v>
-      </c>
-      <c r="D5" s="13" t="n">
-        <f aca="false">C5/(B5/$B$2*$C$2)-1</f>
-        <v>0.297659531906381</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <f aca="false">C5/$I$1</f>
-        <v>65</v>
-      </c>
-      <c r="F5" s="15" t="n">
-        <f aca="false">B5/E5</f>
-        <v>0.769076923076923</v>
-      </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="C7" s="5" t="n">
+        <v>5040</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <f aca="false">C7-ROUND(B7/$B$1*100,0)</f>
+        <v>1707</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <f aca="false">1-F7/$B$1</f>
+        <v>0.338756613756614</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <f aca="false">B7/C7*100</f>
+        <v>0.991865079365079</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <f aca="false">F7*$E$1/100</f>
+        <v>0.991865079365079</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>10200</v>
+      </c>
+      <c r="I7" s="15" t="n">
+        <f aca="false">B7/H7*100</f>
+        <v>0.490098039215686</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="C8" s="16" t="n">
-        <f aca="false">Assumptions!$B$20*Assumptions!$B$21</f>
-        <v>30</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <f aca="false">B8/C8</f>
-        <v>0.166333333333333</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <f aca="false">1-E8/$F$2</f>
-        <v>0.833333333333333</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <f aca="false">Assumptions!$B$17</f>
-        <v>12</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <f aca="false">B9/C9</f>
-        <v>0.8325</v>
-      </c>
-      <c r="F9" s="13" t="n">
-        <f aca="false">1-E9/$F$2</f>
-        <v>0.165831663326653</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B10" s="12" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E10" s="15" t="n">
-        <f aca="false">B10/C10</f>
-        <v>0.499</v>
-      </c>
-      <c r="F10" s="13" t="n">
-        <f aca="false">1-E10/$F$2</f>
-        <v>0.5</v>
-      </c>
+      <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>9.99</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E11" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="15" t="n">
         <f aca="false">B11/C11</f>
-        <v>0.666</v>
-      </c>
-      <c r="F11" s="13" t="n">
-        <f aca="false">1-E11/$F$2</f>
-        <v>0.332665330661323</v>
-      </c>
+        <v>0.999</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <f aca="false">1-D11/$G$4</f>
+        <v>0.334</v>
+      </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <f aca="false">B12/C12</f>
+        <v>0.7495</v>
+      </c>
+      <c r="E12" s="14" t="n">
+        <f aca="false">1-D12/$G$4</f>
+        <v>0.500333333333333</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -2224,16 +2321,139 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <f aca="false">B13/C13</f>
+        <v>0.666333333333333</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <f aca="false">1-D13/$G$4</f>
+        <v>0.555777777777778</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2247,6 +2467,317 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>550</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B7" s="16" t="n">
+        <f aca="false">Assumptions!$B$2</f>
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="17" t="n">
+        <f aca="false">Assumptions!$B$3</f>
+        <v>0.5</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <f aca="false">B8*B4+(1-B8)*B5+B6*B7</f>
+        <v>525</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <f aca="false">B2*B3</f>
+        <v>27500</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B14" s="16" t="n">
+        <f aca="false">Profiles!B2*Profiles!B3</f>
+        <v>20</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <f aca="false">B14*$B$10</f>
+        <v>10500</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <f aca="false">INT(C14/$B$2)</f>
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <f aca="false">D14+15</f>
+        <v>34</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <f aca="false">D14+30</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="16" t="n">
+        <f aca="false">Profiles!C2*Profiles!C3</f>
+        <v>54</v>
+      </c>
+      <c r="C15" s="13" t="n">
+        <f aca="false">B15*$B$10</f>
+        <v>28350</v>
+      </c>
+      <c r="D15" s="2" t="n">
+        <f aca="false">INT(C15/$B$2)</f>
+        <v>51</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <f aca="false">D15+15</f>
+        <v>66</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <f aca="false">D15+30</f>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" s="16" t="n">
+        <f aca="false">Profiles!D2*Profiles!D3</f>
+        <v>156</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <f aca="false">B16*$B$10</f>
+        <v>81900</v>
+      </c>
+      <c r="D16" s="2" t="n">
+        <f aca="false">INT(C16/$B$2)</f>
+        <v>148</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <f aca="false">D16+15</f>
+        <v>163</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <f aca="false">D16+30</f>
+        <v>178</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <f aca="false">Profiles!E2*Profiles!E3</f>
+        <v>360</v>
+      </c>
+      <c r="C17" s="13" t="n">
+        <f aca="false">B17*$B$10</f>
+        <v>189000</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <f aca="false">INT(C17/$B$2)</f>
+        <v>343</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <f aca="false">D17+15</f>
+        <v>358</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <f aca="false">D17+30</f>
+        <v>373</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2264,19 +2795,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -2284,12 +2815,12 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="C2" s="17" t="n">
+      <c r="C2" s="18" t="n">
         <f aca="false">B2/SUM($B$2:$B$5)</f>
         <v>0.533333333333333</v>
       </c>
@@ -2305,12 +2836,12 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="B3" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="18" t="n">
         <f aca="false">B3/SUM($B$2:$B$5)</f>
         <v>0.266666666666667</v>
       </c>
@@ -2326,12 +2857,12 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="18" t="n">
         <f aca="false">B4/SUM($B$2:$B$5)</f>
         <v>0.133333333333333</v>
       </c>
@@ -2347,12 +2878,12 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="18" t="n">
         <f aca="false">B5/SUM($B$2:$B$5)</f>
         <v>0.0666666666666667</v>
       </c>
@@ -2368,7 +2899,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>130</v>
+        <v>153</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -2386,7 +2917,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>131</v>
+        <v>154</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2408,23 +2939,23 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>132</v>
+        <v>155</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>133</v>
+        <v>156</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="3" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="H9" s="5" t="n">
         <v>5</v>
@@ -2432,22 +2963,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>80</v>
-      </c>
-      <c r="C10" s="17" t="n">
+        <v>900</v>
+      </c>
+      <c r="C10" s="18" t="n">
         <f aca="false">B10/SUM($B$10:$B$13)</f>
-        <v>0.8</v>
-      </c>
-      <c r="D10" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D10" s="19" t="n">
         <f aca="false">C10*$H$9</f>
-        <v>4</v>
-      </c>
-      <c r="E10" s="14" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <f aca="false">1/D10</f>
-        <v>0.25</v>
+        <v>0.222222222222222</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -2455,22 +2986,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="C11" s="17" t="n">
+        <v>89</v>
+      </c>
+      <c r="C11" s="18" t="n">
         <f aca="false">B11/SUM($B$10:$B$13)</f>
-        <v>0.14</v>
-      </c>
-      <c r="D11" s="18" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="D11" s="19" t="n">
         <f aca="false">C11*$H$9</f>
-        <v>0.7</v>
-      </c>
-      <c r="E11" s="14" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <f aca="false">1/D11</f>
-        <v>1.42857142857143</v>
+        <v>2.24719101123596</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -2478,22 +3009,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>138</v>
+        <v>161</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C12" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="18" t="n">
         <f aca="false">B12/SUM($B$10:$B$13)</f>
+        <v>0.01</v>
+      </c>
+      <c r="D12" s="19" t="n">
+        <f aca="false">C12*$H$9</f>
         <v>0.05</v>
       </c>
-      <c r="D12" s="18" t="n">
-        <f aca="false">C12*$H$9</f>
-        <v>0.25</v>
-      </c>
-      <c r="E12" s="14" t="n">
+      <c r="E12" s="20" t="n">
         <f aca="false">1/D12</f>
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -2501,22 +3032,22 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>139</v>
+        <v>162</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="18" t="n">
         <f aca="false">B13/SUM($B$10:$B$13)</f>
-        <v>0.01</v>
-      </c>
-      <c r="D13" s="18" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="D13" s="19" t="n">
         <f aca="false">C13*$H$9</f>
-        <v>0.05</v>
-      </c>
-      <c r="E13" s="14" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="E13" s="20" t="n">
         <f aca="false">1/D13</f>
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -2534,7 +3065,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>140</v>
+        <v>163</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -2546,11 +3077,11 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>141</v>
+        <v>164</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="19" t="n">
         <f aca="false">C5*$H$9</f>
         <v>0.333333333333333</v>
       </c>
@@ -2558,174 +3089,6 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="B2" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="D2" s="14" t="n">
-        <f aca="false">C2/B2</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="14" t="n">
-        <f aca="false">C3/B3</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>400</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <f aca="false">C4/B4</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>200</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>1600</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <f aca="false">C5/B5</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B8" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="B10" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="B11" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2743,6 +3106,182 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="20" t="n">
+        <f aca="false">C2/B2</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D3" s="20" t="n">
+        <f aca="false">C3/B3</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>250</v>
+      </c>
+      <c r="D4" s="20" t="n">
+        <f aca="false">C4/B4</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D5" s="20" t="n">
+        <f aca="false">C5/B5</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:N9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2751,7 +3290,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>148</v>
+        <v>172</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -2769,7 +3308,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2803,266 +3342,266 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>151</v>
+        <v>174</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>153</v>
+        <v>176</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>156</v>
+        <v>179</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>158</v>
+        <v>181</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>159</v>
+        <v>182</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>14.9</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="14" t="n">
         <v>0.53</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>0.7</v>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="14" t="n">
         <v>0.79</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="14" t="n">
         <v>0.84</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="14" t="n">
         <v>0.87</v>
       </c>
-      <c r="H5" s="13" t="n">
+      <c r="H5" s="14" t="n">
         <v>0.89</v>
       </c>
-      <c r="I5" s="13" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="K5" s="13" t="n">
+      <c r="I5" s="14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="M5" s="14" t="n">
         <v>0.32</v>
       </c>
-      <c r="L5" s="13" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="M5" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>0.43</v>
+      <c r="N5" s="14" t="n">
+        <v>0.34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>30.8</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="14" t="n">
         <v>0.71</v>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>0.84</v>
       </c>
-      <c r="E6" s="13" t="n">
+      <c r="E6" s="14" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="13" t="n">
+      <c r="F6" s="14" t="n">
         <v>0.93</v>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="G6" s="14" t="n">
         <v>0.95</v>
       </c>
-      <c r="H6" s="13" t="n">
+      <c r="H6" s="14" t="n">
         <v>0.96</v>
       </c>
-      <c r="I6" s="13" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="J6" s="13" t="n">
+      <c r="I6" s="14" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K6" s="14" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="L6" s="14" t="n">
         <v>0.37</v>
       </c>
-      <c r="K6" s="13" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="L6" s="13" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="M6" s="13" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="N6" s="13" t="n">
-        <v>0.56</v>
+      <c r="M6" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N6" s="14" t="n">
+        <v>0.42</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>48.9</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>0.9</v>
       </c>
-      <c r="E7" s="13" t="n">
+      <c r="E7" s="14" t="n">
         <v>0.94</v>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="F7" s="14" t="n">
         <v>0.96</v>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="G7" s="14" t="n">
         <v>0.97</v>
       </c>
-      <c r="H7" s="13" t="n">
+      <c r="H7" s="14" t="n">
         <v>0.98</v>
       </c>
-      <c r="I7" s="13" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="J7" s="13" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="K7" s="13" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="L7" s="13" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="M7" s="13" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="N7" s="13" t="n">
-        <v>0.64</v>
+      <c r="I7" s="14" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="M7" s="14" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N7" s="14" t="n">
+        <v>0.48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>55.4</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="14" t="n">
         <v>0.83</v>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>0.92</v>
       </c>
-      <c r="E8" s="13" t="n">
+      <c r="E8" s="14" t="n">
         <v>0.95</v>
       </c>
-      <c r="F8" s="13" t="n">
+      <c r="F8" s="14" t="n">
         <v>0.97</v>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="G8" s="14" t="n">
         <v>0.98</v>
       </c>
-      <c r="H8" s="13" t="n">
+      <c r="H8" s="14" t="n">
         <v>0.99</v>
       </c>
-      <c r="I8" s="13" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="N8" s="13" t="n">
-        <v>0.66</v>
+      <c r="I8" s="14" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="K8" s="14" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="L8" s="14" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="M8" s="14" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="N8" s="14" t="n">
+        <v>0.49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>90.9</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="14" t="n">
         <v>0.9</v>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>0.96</v>
       </c>
-      <c r="E9" s="13" t="n">
+      <c r="E9" s="14" t="n">
         <v>0.98</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="14" t="n">
         <v>0.99</v>
       </c>
-      <c r="G9" s="13" t="n">
+      <c r="G9" s="14" t="n">
         <v>0.99</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="13" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="J9" s="13" t="n">
+      <c r="I9" s="14" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N9" s="14" t="n">
         <v>0.55</v>
-      </c>
-      <c r="K9" s="13" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="L9" s="13" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="M9" s="13" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="N9" s="13" t="n">
-        <v>0.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>